<commit_message>
Sorted all Verdant forest opponents, created custom sprites for gym leaders
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68643065-5D0E-4C7A-B8A3-5AE080410DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9069453-FFAC-49B0-ADD7-CE3C918E8D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="12645" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="43200" windowHeight="11295" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -81,6 +81,15 @@
   </si>
   <si>
     <t>https://eeveeexpo.com/resources/404/</t>
+  </si>
+  <si>
+    <t>Kanto Gym Leader Sprites</t>
+  </si>
+  <si>
+    <t>Drawnamu</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/drawnamu/art/Kanto-gym-leaders-Elite-4-graphical-evolution-624351384</t>
   </si>
 </sst>
 </file>
@@ -125,9 +134,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -463,11 +475,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="44.5703125" customWidth="1"/>
-    <col min="3" max="3" width="38.85546875" customWidth="1"/>
+    <col min="3" max="3" width="93.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -536,6 +548,17 @@
       </c>
       <c r="C7" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprite updates: Added Rival overworld and in battle sprites
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9069453-FFAC-49B0-ADD7-CE3C918E8D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA03F55B-38E8-4795-A68F-C6ACBDC3095D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="43200" windowHeight="11295" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -90,6 +90,25 @@
   </si>
   <si>
     <t>https://www.deviantart.com/drawnamu/art/Kanto-gym-leaders-Elite-4-graphical-evolution-624351384</t>
+  </si>
+  <si>
+    <t>Tobalcr</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/thecubberx/art/URBAIN-AND-TAUNIE-SPRITES-1199732630</t>
+  </si>
+  <si>
+    <t>THEcubberx</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/tobalcr/art/URBAIN-URBI-FROM-POKEMON-ZA-OVERWORLD-BW-STYLE-1244035276
+https://www.deviantart.com/tobalcr/art/TAUNIE-MUNI-FROM-POKEMON-ZA-OVERWORLD-BW-STYLE-1244034913</t>
+  </si>
+  <si>
+    <t>Urbain &amp; Taunie Overworld Sprites</t>
+  </si>
+  <si>
+    <t>Urbain &amp; Taunie In-Battle Sprites</t>
   </si>
 </sst>
 </file>
@@ -475,11 +494,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="44.5703125" customWidth="1"/>
-    <col min="3" max="3" width="93.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="109.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -561,10 +580,33 @@
         <v>17</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://www.reddit.com/r/PokemonRMXP/" xr:uid="{484AF3F9-A79A-44A4-BE84-81893A8B5A0F}"/>
     <hyperlink ref="B3" r:id="rId2" display="https://www.reddit.com/user/New_Personality_9208/" xr:uid="{B6FC823D-A351-4968-90C5-AB0A9D22DCC7}"/>
+    <hyperlink ref="B10" r:id="rId3" display="https://www.deviantart.com/thecubberx/gallery" xr:uid="{1CE16580-A4E8-4E2A-8B7A-6EEC4BA2FD45}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Assets: Downloaded 300 card sleeve images to use
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA03F55B-38E8-4795-A68F-C6ACBDC3095D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A483B850-49AA-4960-9B9A-12A5D7C89EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="43200" windowHeight="11295" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -109,6 +109,15 @@
   </si>
   <si>
     <t>Urbain &amp; Taunie In-Battle Sprites</t>
+  </si>
+  <si>
+    <t>https://pokemon-sleeve-database.com/</t>
+  </si>
+  <si>
+    <t>LittleJoeJoe</t>
+  </si>
+  <si>
+    <t>All Scanned Pokemon Sleeves</t>
   </si>
 </sst>
 </file>
@@ -494,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="44.5703125" customWidth="1"/>
@@ -602,6 +611,17 @@
         <v>19</v>
       </c>
     </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://www.reddit.com/r/PokemonRMXP/" xr:uid="{484AF3F9-A79A-44A4-BE84-81893A8B5A0F}"/>

</xml_diff>

<commit_message>
Assets: Added more sleeves
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A483B850-49AA-4960-9B9A-12A5D7C89EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E960E02-6E91-4345-B4C1-629219221CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="43200" windowHeight="11295" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="11970" windowHeight="15585" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -117,7 +117,25 @@
     <t>LittleJoeJoe</t>
   </si>
   <si>
-    <t>All Scanned Pokemon Sleeves</t>
+    <t>Sleeping Pokemon Sleeve art</t>
+  </si>
+  <si>
+    <t>https://x.com/hyogonosuke</t>
+  </si>
+  <si>
+    <t>hyogonosuke</t>
+  </si>
+  <si>
+    <t>https://www.elitefourum.com/u/koala/activity/topics</t>
+  </si>
+  <si>
+    <t>Koala</t>
+  </si>
+  <si>
+    <t>Pokemon TCG Pocket full art sleeves</t>
+  </si>
+  <si>
+    <t>IRL Scanned Pokemon Sleeves</t>
   </si>
 </sst>
 </file>
@@ -503,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="44.5703125" customWidth="1"/>
@@ -613,13 +631,35 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
         <v>25</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sprites: Added 36 new trainer sprites and a bunch of NPCs
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E960E02-6E91-4345-B4C1-629219221CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14CED6E-8685-432D-B2B5-C729BD2B1124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="11970" windowHeight="15585" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -136,6 +136,66 @@
   </si>
   <si>
     <t>IRL Scanned Pokemon Sleeves</t>
+  </si>
+  <si>
+    <t>Backers in battle sprite</t>
+  </si>
+  <si>
+    <t>AurumDeluxe</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/aurumdeluxe</t>
+  </si>
+  <si>
+    <t>DiegoWT</t>
+  </si>
+  <si>
+    <t>Credits:
+Artist:
+Taiga
+Some sprites use assets/colours/inspiration from:
+DiegoWT
+Neo-Spriteman
+Vanilla Sunshine
+AtomicReactor
+PurpleZaffre
+izzyvivious
+Tebited
+Sprites used:
+PizzaSun  - Lysandre,Calem,Serena
+izzyvicious  - AZ
+Wolfgang62 - Viola, Diantha
+Somersault - Ramos</t>
+  </si>
+  <si>
+    <t>https://eeveeexpo.com/resources/1057/</t>
+  </si>
+  <si>
+    <t>RuinManiacF sprite</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/kingtapir/gallery</t>
+  </si>
+  <si>
+    <t>KingTapir, KyleDove &amp; JaneJewel</t>
+  </si>
+  <si>
+    <t>TeenagerM&amp;F, Neckbeard, XY, USUM, ORAS overworld sprites</t>
+  </si>
+  <si>
+    <t>Team Skull M/F Overworld Sprite</t>
+  </si>
+  <si>
+    <t>Team Skull M/F In Battle Sprite</t>
+  </si>
+  <si>
+    <t>Mid117</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/diegowt/art/Team-Skull-female-grunt-1020343907</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/mid117/art/Pokemon-Sun-and-Moon-Team-Skull-Grunts-Sprite-657950401</t>
   </si>
 </sst>
 </file>
@@ -180,11 +240,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -521,14 +584,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="44.5703125" customWidth="1"/>
-    <col min="3" max="3" width="109.7109375" customWidth="1"/>
+    <col min="1" max="1" width="51.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.5546875" customWidth="1"/>
+    <col min="3" max="3" width="109.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -539,7 +603,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -550,7 +614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -561,7 +625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -572,7 +636,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -580,7 +644,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -588,7 +652,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -596,7 +660,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -607,7 +671,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -618,7 +682,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -629,7 +693,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -640,7 +704,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -651,7 +715,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -660,6 +724,61 @@
       </c>
       <c r="C13" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -667,6 +786,8 @@
     <hyperlink ref="C3" r:id="rId1" display="https://www.reddit.com/r/PokemonRMXP/" xr:uid="{484AF3F9-A79A-44A4-BE84-81893A8B5A0F}"/>
     <hyperlink ref="B3" r:id="rId2" display="https://www.reddit.com/user/New_Personality_9208/" xr:uid="{B6FC823D-A351-4968-90C5-AB0A9D22DCC7}"/>
     <hyperlink ref="B10" r:id="rId3" display="https://www.deviantart.com/thecubberx/gallery" xr:uid="{1CE16580-A4E8-4E2A-8B7A-6EEC4BA2FD45}"/>
+    <hyperlink ref="B14" r:id="rId4" display="https://www.deviantart.com/aurumdeluxe" xr:uid="{DF54BD18-078B-4049-BEBB-106BDA490062}"/>
+    <hyperlink ref="B17" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Debug: Fixed dozens of issues with UI and other bugs
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14CED6E-8685-432D-B2B5-C729BD2B1124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92BFBBB-58FC-4020-9CB7-2A89EE1750C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -196,6 +196,15 @@
   </si>
   <si>
     <t>https://www.deviantart.com/mid117/art/Pokemon-Sun-and-Moon-Team-Skull-Grunts-Sprite-657950401</t>
+  </si>
+  <si>
+    <t>XY, USUM, ORAS in battle sprites</t>
+  </si>
+  <si>
+    <t>Kyle-Dove</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/kyle-dove/gallery</t>
   </si>
 </sst>
 </file>
@@ -584,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="51.109375" bestFit="1" customWidth="1"/>
@@ -750,34 +759,45 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" t="s">
-        <v>41</v>
+        <v>48</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>44</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>45</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>47</v>
       </c>
     </row>
@@ -787,7 +807,7 @@
     <hyperlink ref="B3" r:id="rId2" display="https://www.reddit.com/user/New_Personality_9208/" xr:uid="{B6FC823D-A351-4968-90C5-AB0A9D22DCC7}"/>
     <hyperlink ref="B10" r:id="rId3" display="https://www.deviantart.com/thecubberx/gallery" xr:uid="{1CE16580-A4E8-4E2A-8B7A-6EEC4BA2FD45}"/>
     <hyperlink ref="B14" r:id="rId4" display="https://www.deviantart.com/aurumdeluxe" xr:uid="{DF54BD18-078B-4049-BEBB-106BDA490062}"/>
-    <hyperlink ref="B17" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
+    <hyperlink ref="B18" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>